<commit_message>
Apply final review: test fix, corrected note and README, license
Fix the SQL/Python test for different date resolutions, pin package
versions, drop windows before the ECB meeting calendar from the no-ECB check,
correct the sample description (March-December 2020), qualify the
interpretation in the note, add the MIT license and the review response.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/excel/global_markets_monitor.xlsx
+++ b/outputs/excel/global_markets_monitor.xlsx
@@ -4052,22 +4052,22 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>1.9192</v>
+        <v>1.9382</v>
       </c>
       <c r="E14" t="n">
-        <v>1.1195</v>
+        <v>1.1222</v>
       </c>
       <c r="F14" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>3.7606</v>
+        <v>3.7841</v>
       </c>
       <c r="H14" t="n">
-        <v>0.08649999999999999</v>
+        <v>0.08409999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15">
@@ -4085,22 +4085,22 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>1.7985</v>
+        <v>1.8205</v>
       </c>
       <c r="E15" t="n">
-        <v>1.3621</v>
+        <v>1.3681</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.442</v>
+        <v>-0.4298</v>
       </c>
       <c r="G15" t="n">
-        <v>4.039</v>
+        <v>4.0707</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1867</v>
+        <v>0.1833</v>
       </c>
       <c r="I15" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16">
@@ -4118,22 +4118,22 @@
         <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>3.8216</v>
+        <v>3.8433</v>
       </c>
       <c r="E16" t="n">
-        <v>2.1207</v>
+        <v>2.125</v>
       </c>
       <c r="F16" t="n">
-        <v>0.3334</v>
+        <v>0.348</v>
       </c>
       <c r="G16" t="n">
-        <v>7.3098</v>
+        <v>7.3386</v>
       </c>
       <c r="H16" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17">
@@ -4151,22 +4151,22 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0025</v>
+        <v>0.0026</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0039</v>
+        <v>-0.004</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0045</v>
+        <v>0.0044</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9043</v>
+        <v>0.9283</v>
       </c>
       <c r="I17" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18">
@@ -4184,22 +4184,22 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
       <c r="E18" t="n">
         <v>0.0047</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0043</v>
+        <v>-0.0044</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0113</v>
+        <v>0.0111</v>
       </c>
       <c r="H18" t="n">
-        <v>0.459</v>
+        <v>0.476</v>
       </c>
       <c r="I18" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19">
@@ -4217,22 +4217,22 @@
         <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0139</v>
+        <v>0.0138</v>
       </c>
       <c r="E19" t="n">
         <v>0.0083</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0275</v>
+        <v>0.0274</v>
       </c>
       <c r="H19" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.097</v>
       </c>
       <c r="I19" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20">
@@ -4250,22 +4250,22 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.5384</v>
+        <v>-0.5405</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1517</v>
+        <v>0.1519</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.788</v>
+        <v>-0.7904</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.2888</v>
+        <v>-0.2906</v>
       </c>
       <c r="H20" t="n">
         <v>0.0004</v>
       </c>
       <c r="I20" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21">
@@ -4283,22 +4283,22 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.6815</v>
+        <v>-0.6830000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2431</v>
+        <v>0.2432</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.0814</v>
+        <v>-1.0831</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.2816</v>
+        <v>-0.283</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0051</v>
+        <v>0.005</v>
       </c>
       <c r="I21" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22">
@@ -4316,22 +4316,22 @@
         <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.3368</v>
+        <v>-0.337</v>
       </c>
       <c r="E22" t="n">
         <v>0.2767</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.792</v>
+        <v>-0.7922</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1184</v>
+        <v>0.1182</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2236</v>
+        <v>0.2233</v>
       </c>
       <c r="I22" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23">
@@ -4349,22 +4349,22 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>4.1208</v>
+        <v>4.15</v>
       </c>
       <c r="E23" t="n">
-        <v>1.8361</v>
+        <v>1.8385</v>
       </c>
       <c r="F23" t="n">
-        <v>1.1007</v>
+        <v>1.1259</v>
       </c>
       <c r="G23" t="n">
-        <v>7.1409</v>
+        <v>7.174</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0248</v>
+        <v>0.024</v>
       </c>
       <c r="I23" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24">
@@ -4382,22 +4382,22 @@
         <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>3.5612</v>
+        <v>3.6063</v>
       </c>
       <c r="E24" t="n">
-        <v>2.4103</v>
+        <v>2.4162</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.4034</v>
+        <v>-0.368</v>
       </c>
       <c r="G24" t="n">
-        <v>7.5257</v>
+        <v>7.5806</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1395</v>
+        <v>0.1356</v>
       </c>
       <c r="I24" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25">
@@ -4415,22 +4415,22 @@
         <v>5</v>
       </c>
       <c r="D25" t="n">
-        <v>5.6023</v>
+        <v>5.6354</v>
       </c>
       <c r="E25" t="n">
-        <v>2.6676</v>
+        <v>2.675</v>
       </c>
       <c r="F25" t="n">
-        <v>1.2145</v>
+        <v>1.2354</v>
       </c>
       <c r="G25" t="n">
-        <v>9.9901</v>
+        <v>10.0354</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0357</v>
+        <v>0.0351</v>
       </c>
       <c r="I25" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26">

</xml_diff>